<commit_message>
Add Visits + one-to-many Treatment Plans; follow-up chasing workflow (W12); reverse T4
</commit_message>
<xml_diff>
--- a/docs/ProstaCare_Schema_V3_proposed.xlsx
+++ b/docs/ProstaCare_Schema_V3_proposed.xlsx
@@ -34,6 +34,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QoL_Assessments" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Healthcare_Contacts" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrals" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Treatment_Plans" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -47,7 +49,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -99,6 +101,11 @@
       <b val="1"/>
       <color rgb="001D4F91"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001D4F91"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -320,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -393,6 +400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1062,6 +1070,123 @@
       <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Terminology alignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t>Round 2 — visits &amp; repeat treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Visits (NEW sheet)</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>Every attendance recorded: date, type, disease state, outcome, next visit due</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>Patient returns repeatedly; drives follow-up tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Treatment_Plans (NEW sheet)</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>Treatment plan becomes ONE-TO-MANY (a dated version per line of therapy)</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>A new plan is agreed at progression / toxicity</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Treatment_Entry</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>treatment_intent, mdt_status, date_of_mdt_review moved to Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>They belong to a plan version, not to the patient</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Dated sheets</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>OPTIONAL visit_id link on PSA, labs, clinical, treatment, AEs, journey</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Groups everything captured at one visit; still valid without it</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>next_visit_due_date + disease_state_at_visit drive the 'follow-up overdue' nudge</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>Protocol intervals by disease state (pathway panel 5)</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D376"/>
+  <dimension ref="A1:D411"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1099,7 +1224,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -8555,6 +8679,706 @@
       <c r="D376" s="20" t="inlineStr">
         <is>
           <t>PROPOSED (v3) — pending clinical sign-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B377" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C377" s="20" t="inlineStr">
+        <is>
+          <t>First consultation</t>
+        </is>
+      </c>
+      <c r="D377" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B378" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C378" s="20" t="inlineStr">
+        <is>
+          <t>Follow-up review</t>
+        </is>
+      </c>
+      <c r="D378" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B379" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C379" s="20" t="inlineStr">
+        <is>
+          <t>Treatment / day-care</t>
+        </is>
+      </c>
+      <c r="D379" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B380" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C380" s="20" t="inlineStr">
+        <is>
+          <t>MDT review</t>
+        </is>
+      </c>
+      <c r="D380" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B381" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C381" s="20" t="inlineStr">
+        <is>
+          <t>Investigation only</t>
+        </is>
+      </c>
+      <c r="D381" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B382" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C382" s="20" t="inlineStr">
+        <is>
+          <t>Emergency / unplanned</t>
+        </is>
+      </c>
+      <c r="D382" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="20" t="inlineStr">
+        <is>
+          <t>visitType</t>
+        </is>
+      </c>
+      <c r="B383" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C383" s="20" t="inlineStr">
+        <is>
+          <t>Telemedicine</t>
+        </is>
+      </c>
+      <c r="D383" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B384" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C384" s="20" t="inlineStr">
+        <is>
+          <t>Localized — on active surveillance</t>
+        </is>
+      </c>
+      <c r="D384" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B385" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C385" s="20" t="inlineStr">
+        <is>
+          <t>Localized / locally advanced — on curative treatment</t>
+        </is>
+      </c>
+      <c r="D385" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B386" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C386" s="20" t="inlineStr">
+        <is>
+          <t>mHSPC (metastatic hormone-sensitive)</t>
+        </is>
+      </c>
+      <c r="D386" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B387" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C387" s="20" t="inlineStr">
+        <is>
+          <t>mCRPC (metastatic castration-resistant)</t>
+        </is>
+      </c>
+      <c r="D387" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B388" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C388" s="20" t="inlineStr">
+        <is>
+          <t>On radioligand therapy (Pluvicto)</t>
+        </is>
+      </c>
+      <c r="D388" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="20" t="inlineStr">
+        <is>
+          <t>diseaseStateAtVisit</t>
+        </is>
+      </c>
+      <c r="B389" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C389" s="20" t="inlineStr">
+        <is>
+          <t>Long-term survivor / surveillance</t>
+        </is>
+      </c>
+      <c r="D389" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B390" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C390" s="20" t="inlineStr">
+        <is>
+          <t>Continue current plan</t>
+        </is>
+      </c>
+      <c r="D390" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B391" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C391" s="20" t="inlineStr">
+        <is>
+          <t>Treatment plan changed</t>
+        </is>
+      </c>
+      <c r="D391" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B392" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C392" s="20" t="inlineStr">
+        <is>
+          <t>Referred to another service</t>
+        </is>
+      </c>
+      <c r="D392" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B393" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C393" s="20" t="inlineStr">
+        <is>
+          <t>Admitted</t>
+        </is>
+      </c>
+      <c r="D393" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B394" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C394" s="20" t="inlineStr">
+        <is>
+          <t>Discharged from follow-up</t>
+        </is>
+      </c>
+      <c r="D394" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="20" t="inlineStr">
+        <is>
+          <t>visitOutcome</t>
+        </is>
+      </c>
+      <c r="B395" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C395" s="20" t="inlineStr">
+        <is>
+          <t>Deceased</t>
+        </is>
+      </c>
+      <c r="D395" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="20" t="inlineStr">
+        <is>
+          <t>lineOfTherapy</t>
+        </is>
+      </c>
+      <c r="B396" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C396" s="20" t="inlineStr">
+        <is>
+          <t>1st line</t>
+        </is>
+      </c>
+      <c r="D396" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="20" t="inlineStr">
+        <is>
+          <t>lineOfTherapy</t>
+        </is>
+      </c>
+      <c r="B397" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C397" s="20" t="inlineStr">
+        <is>
+          <t>2nd line</t>
+        </is>
+      </c>
+      <c r="D397" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="20" t="inlineStr">
+        <is>
+          <t>lineOfTherapy</t>
+        </is>
+      </c>
+      <c r="B398" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C398" s="20" t="inlineStr">
+        <is>
+          <t>3rd line</t>
+        </is>
+      </c>
+      <c r="D398" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="20" t="inlineStr">
+        <is>
+          <t>lineOfTherapy</t>
+        </is>
+      </c>
+      <c r="B399" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C399" s="20" t="inlineStr">
+        <is>
+          <t>4th line or later</t>
+        </is>
+      </c>
+      <c r="D399" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="20" t="inlineStr">
+        <is>
+          <t>planStatus</t>
+        </is>
+      </c>
+      <c r="B400" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C400" s="20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D400" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="20" t="inlineStr">
+        <is>
+          <t>planStatus</t>
+        </is>
+      </c>
+      <c r="B401" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C401" s="20" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="D401" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="20" t="inlineStr">
+        <is>
+          <t>planStatus</t>
+        </is>
+      </c>
+      <c r="B402" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C402" s="20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D402" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="20" t="inlineStr">
+        <is>
+          <t>planStatus</t>
+        </is>
+      </c>
+      <c r="B403" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C403" s="20" t="inlineStr">
+        <is>
+          <t>Stopped — toxicity</t>
+        </is>
+      </c>
+      <c r="D403" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="20" t="inlineStr">
+        <is>
+          <t>planStatus</t>
+        </is>
+      </c>
+      <c r="B404" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C404" s="20" t="inlineStr">
+        <is>
+          <t>Stopped — patient choice</t>
+        </is>
+      </c>
+      <c r="D404" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B405" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C405" s="20" t="inlineStr">
+        <is>
+          <t>Initial plan</t>
+        </is>
+      </c>
+      <c r="D405" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B406" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C406" s="20" t="inlineStr">
+        <is>
+          <t>Disease progression</t>
+        </is>
+      </c>
+      <c r="D406" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B407" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C407" s="20" t="inlineStr">
+        <is>
+          <t>Toxicity / intolerance</t>
+        </is>
+      </c>
+      <c r="D407" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B408" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C408" s="20" t="inlineStr">
+        <is>
+          <t>Patient preference</t>
+        </is>
+      </c>
+      <c r="D408" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B409" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C409" s="20" t="inlineStr">
+        <is>
+          <t>Access / affordability</t>
+        </is>
+      </c>
+      <c r="D409" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B410" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C410" s="20" t="inlineStr">
+        <is>
+          <t>Completed planned course</t>
+        </is>
+      </c>
+      <c r="D410" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="20" t="inlineStr">
+        <is>
+          <t>reasonForPlanChange</t>
+        </is>
+      </c>
+      <c r="B411" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C411" s="20" t="inlineStr">
+        <is>
+          <t>Comorbidity</t>
+        </is>
+      </c>
+      <c r="D411" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3) — visits &amp; treatment plans</t>
         </is>
       </c>
     </row>
@@ -40785,6 +41609,92 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>Visits — PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Repeating rows — the patient returns many times. Reuse the same Unique Patient Code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Unique Patient Code</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Visit Date</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Visit Type</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Seen By (clinician)</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Disease State at Visit</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Reason for Visit</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>Visit Outcome</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Next Visit Due</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -41164,6 +42074,92 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>Treatment Plans — PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Repeating rows — the patient returns many times. Reuse the same Unique Patient Code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Unique Patient Code</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Plan Date</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Line of Therapy</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Treatment Intent</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>MDT / Tumour Board Status</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Date of MDT Review</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>Reason for This Plan</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Plan Status</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Plan Summary</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -43202,7 +44198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -46590,9 +47586,9 @@
         </is>
       </c>
       <c r="K59" s="14" t="n"/>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Existing (v2)</t>
+      <c r="L59" s="20" t="inlineStr">
+        <is>
+          <t>SUPERSEDED (v3) → moved to Treatment_Plans (now one-to-many)</t>
         </is>
       </c>
     </row>
@@ -46648,9 +47644,9 @@
         </is>
       </c>
       <c r="K60" s="14" t="n"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Existing (v2)</t>
+      <c r="L60" s="20" t="inlineStr">
+        <is>
+          <t>SUPERSEDED (v3) → moved to Treatment_Plans (now one-to-many)</t>
         </is>
       </c>
     </row>
@@ -46706,9 +47702,9 @@
         </is>
       </c>
       <c r="K61" s="14" t="n"/>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>Existing (v2)</t>
+      <c r="L61" s="20" t="inlineStr">
+        <is>
+          <t>SUPERSEDED (v3) → moved to Treatment_Plans (now one-to-many)</t>
         </is>
       </c>
     </row>
@@ -52333,6 +53329,1470 @@
         </is>
       </c>
       <c r="L156" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B157" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C157" s="20" t="inlineStr">
+        <is>
+          <t>patient_code</t>
+        </is>
+      </c>
+      <c r="D157" s="20" t="inlineStr">
+        <is>
+          <t>Unique Patient Code</t>
+        </is>
+      </c>
+      <c r="E157" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F157" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row key</t>
+        </is>
+      </c>
+      <c r="G157" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H157" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I157" s="20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J157" s="20" t="inlineStr"/>
+      <c r="K157" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L157" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B158" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C158" s="20" t="inlineStr">
+        <is>
+          <t>visit_date</t>
+        </is>
+      </c>
+      <c r="D158" s="20" t="inlineStr">
+        <is>
+          <t>Visit Date</t>
+        </is>
+      </c>
+      <c r="E158" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F158" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G158" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="H158" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I158" s="20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J158" s="20" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="K158" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L158" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B159" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C159" s="20" t="inlineStr">
+        <is>
+          <t>visit_type</t>
+        </is>
+      </c>
+      <c r="D159" s="20" t="inlineStr">
+        <is>
+          <t>Visit Type</t>
+        </is>
+      </c>
+      <c r="E159" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F159" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G159" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H159" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I159" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J159" s="20" t="inlineStr">
+        <is>
+          <t>First consultation | Follow-up review | Treatment / day-care | MDT review | Investigation only | Emergency / unplanned | Telemedicine</t>
+        </is>
+      </c>
+      <c r="K159" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L159" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B160" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C160" s="20" t="inlineStr">
+        <is>
+          <t>seen_by</t>
+        </is>
+      </c>
+      <c r="D160" s="20" t="inlineStr">
+        <is>
+          <t>Seen By (clinician)</t>
+        </is>
+      </c>
+      <c r="E160" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F160" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G160" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H160" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I160" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J160" s="20" t="inlineStr"/>
+      <c r="K160" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L160" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B161" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C161" s="20" t="inlineStr">
+        <is>
+          <t>disease_state_at_visit</t>
+        </is>
+      </c>
+      <c r="D161" s="20" t="inlineStr">
+        <is>
+          <t>Disease State at Visit</t>
+        </is>
+      </c>
+      <c r="E161" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F161" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G161" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H161" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I161" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J161" s="20" t="inlineStr">
+        <is>
+          <t>Localized — on active surveillance | Localized / locally advanced — on curative treatment | mHSPC (metastatic hormone-sensitive) | mCRPC (metastatic castration-resistant) | On radioligand therapy (Pluvicto) | Long-term survivor / surveillance</t>
+        </is>
+      </c>
+      <c r="K161" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L161" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B162" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C162" s="20" t="inlineStr">
+        <is>
+          <t>visit_reason</t>
+        </is>
+      </c>
+      <c r="D162" s="20" t="inlineStr">
+        <is>
+          <t>Reason for Visit</t>
+        </is>
+      </c>
+      <c r="E162" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F162" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G162" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H162" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I162" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J162" s="20" t="inlineStr"/>
+      <c r="K162" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L162" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B163" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C163" s="20" t="inlineStr">
+        <is>
+          <t>visit_outcome</t>
+        </is>
+      </c>
+      <c r="D163" s="20" t="inlineStr">
+        <is>
+          <t>Visit Outcome</t>
+        </is>
+      </c>
+      <c r="E163" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F163" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G163" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H163" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I163" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J163" s="20" t="inlineStr">
+        <is>
+          <t>Continue current plan | Treatment plan changed | Referred to another service | Admitted | Discharged from follow-up | Deceased</t>
+        </is>
+      </c>
+      <c r="K163" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L163" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B164" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C164" s="20" t="inlineStr">
+        <is>
+          <t>next_visit_due_date</t>
+        </is>
+      </c>
+      <c r="D164" s="20" t="inlineStr">
+        <is>
+          <t>Next Visit Due</t>
+        </is>
+      </c>
+      <c r="E164" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F164" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G164" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="H164" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I164" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J164" s="20" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="K164" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L164" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="B165" s="20" t="inlineStr">
+        <is>
+          <t>Visits</t>
+        </is>
+      </c>
+      <c r="C165" s="20" t="inlineStr">
+        <is>
+          <t>visit_notes</t>
+        </is>
+      </c>
+      <c r="D165" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E165" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F165" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G165" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H165" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I165" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J165" s="20" t="inlineStr"/>
+      <c r="K165" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L165" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B166" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C166" s="20" t="inlineStr">
+        <is>
+          <t>patient_code</t>
+        </is>
+      </c>
+      <c r="D166" s="20" t="inlineStr">
+        <is>
+          <t>Unique Patient Code</t>
+        </is>
+      </c>
+      <c r="E166" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F166" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row key</t>
+        </is>
+      </c>
+      <c r="G166" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H166" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I166" s="20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J166" s="20" t="inlineStr"/>
+      <c r="K166" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L166" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B167" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C167" s="20" t="inlineStr">
+        <is>
+          <t>plan_date</t>
+        </is>
+      </c>
+      <c r="D167" s="20" t="inlineStr">
+        <is>
+          <t>Plan Date</t>
+        </is>
+      </c>
+      <c r="E167" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F167" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G167" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="H167" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I167" s="20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J167" s="20" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="K167" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L167" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B168" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C168" s="20" t="inlineStr">
+        <is>
+          <t>line_of_therapy</t>
+        </is>
+      </c>
+      <c r="D168" s="20" t="inlineStr">
+        <is>
+          <t>Line of Therapy</t>
+        </is>
+      </c>
+      <c r="E168" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F168" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G168" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H168" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I168" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J168" s="20" t="inlineStr">
+        <is>
+          <t>1st line | 2nd line | 3rd line | 4th line or later</t>
+        </is>
+      </c>
+      <c r="K168" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L168" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B169" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C169" s="20" t="inlineStr">
+        <is>
+          <t>treatment_intent</t>
+        </is>
+      </c>
+      <c r="D169" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Intent</t>
+        </is>
+      </c>
+      <c r="E169" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F169" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G169" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H169" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I169" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J169" s="20" t="inlineStr">
+        <is>
+          <t>treatmentIntent</t>
+        </is>
+      </c>
+      <c r="K169" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L169" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B170" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C170" s="20" t="inlineStr">
+        <is>
+          <t>mdt_tumour_board_status</t>
+        </is>
+      </c>
+      <c r="D170" s="20" t="inlineStr">
+        <is>
+          <t>MDT / Tumour Board Status</t>
+        </is>
+      </c>
+      <c r="E170" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F170" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G170" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H170" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I170" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J170" s="20" t="inlineStr">
+        <is>
+          <t>mdtStatus</t>
+        </is>
+      </c>
+      <c r="K170" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L170" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B171" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C171" s="20" t="inlineStr">
+        <is>
+          <t>date_of_mdt_review</t>
+        </is>
+      </c>
+      <c r="D171" s="20" t="inlineStr">
+        <is>
+          <t>Date of MDT Review</t>
+        </is>
+      </c>
+      <c r="E171" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F171" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G171" s="20" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="H171" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I171" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J171" s="20" t="inlineStr">
+        <is>
+          <t>yyyy-mm-dd</t>
+        </is>
+      </c>
+      <c r="K171" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L171" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B172" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C172" s="20" t="inlineStr">
+        <is>
+          <t>reason_for_plan_change</t>
+        </is>
+      </c>
+      <c r="D172" s="20" t="inlineStr">
+        <is>
+          <t>Reason for This Plan</t>
+        </is>
+      </c>
+      <c r="E172" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F172" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G172" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H172" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I172" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J172" s="20" t="inlineStr">
+        <is>
+          <t>Initial plan | Disease progression | Toxicity / intolerance | Patient preference | Access / affordability | Completed planned course | Comorbidity</t>
+        </is>
+      </c>
+      <c r="K172" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L172" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B173" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C173" s="20" t="inlineStr">
+        <is>
+          <t>plan_status</t>
+        </is>
+      </c>
+      <c r="D173" s="20" t="inlineStr">
+        <is>
+          <t>Plan Status</t>
+        </is>
+      </c>
+      <c r="E173" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F173" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G173" s="20" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="H173" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I173" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J173" s="20" t="inlineStr">
+        <is>
+          <t>Active | Superseded | Completed | Stopped — toxicity | Stopped — patient choice</t>
+        </is>
+      </c>
+      <c r="K173" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L173" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Plans</t>
+        </is>
+      </c>
+      <c r="B174" s="20" t="inlineStr">
+        <is>
+          <t>Treatment Plans</t>
+        </is>
+      </c>
+      <c r="C174" s="20" t="inlineStr">
+        <is>
+          <t>plan_summary</t>
+        </is>
+      </c>
+      <c r="D174" s="20" t="inlineStr">
+        <is>
+          <t>Plan Summary</t>
+        </is>
+      </c>
+      <c r="E174" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F174" s="20" t="inlineStr">
+        <is>
+          <t>Repeating row field</t>
+        </is>
+      </c>
+      <c r="G174" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H174" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I174" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J174" s="20" t="inlineStr"/>
+      <c r="K174" s="20" t="inlineStr">
+        <is>
+          <t>Visits recur; each treatment plan is a dated version.</t>
+        </is>
+      </c>
+      <c r="L174" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="20" t="inlineStr">
+        <is>
+          <t>PSA_History</t>
+        </is>
+      </c>
+      <c r="B175" s="20" t="inlineStr">
+        <is>
+          <t>PSA History &amp; Trend</t>
+        </is>
+      </c>
+      <c r="C175" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D175" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E175" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F175" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G175" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H175" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I175" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J175" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K175" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L175" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="20" t="inlineStr">
+        <is>
+          <t>Clinical_Entry</t>
+        </is>
+      </c>
+      <c r="B176" s="20" t="inlineStr">
+        <is>
+          <t>Workbook Linkage</t>
+        </is>
+      </c>
+      <c r="C176" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D176" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E176" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F176" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G176" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H176" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I176" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J176" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K176" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L176" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="20" t="inlineStr">
+        <is>
+          <t>Treatment_Entry</t>
+        </is>
+      </c>
+      <c r="B177" s="20" t="inlineStr">
+        <is>
+          <t>Workbook Linkage</t>
+        </is>
+      </c>
+      <c r="C177" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D177" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E177" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F177" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G177" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H177" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I177" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J177" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K177" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L177" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="20" t="inlineStr">
+        <is>
+          <t>Journey_Events</t>
+        </is>
+      </c>
+      <c r="B178" s="20" t="inlineStr">
+        <is>
+          <t>Patient Journey</t>
+        </is>
+      </c>
+      <c r="C178" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D178" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E178" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F178" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G178" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H178" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I178" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J178" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K178" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L178" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="20" t="inlineStr">
+        <is>
+          <t>Lab_Results</t>
+        </is>
+      </c>
+      <c r="B179" s="20" t="inlineStr">
+        <is>
+          <t>Lab Results</t>
+        </is>
+      </c>
+      <c r="C179" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D179" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E179" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F179" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G179" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H179" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I179" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J179" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K179" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L179" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="20" t="inlineStr">
+        <is>
+          <t>Adverse_Events</t>
+        </is>
+      </c>
+      <c r="B180" s="20" t="inlineStr">
+        <is>
+          <t>Adverse Events</t>
+        </is>
+      </c>
+      <c r="C180" s="20" t="inlineStr">
+        <is>
+          <t>visit_id</t>
+        </is>
+      </c>
+      <c r="D180" s="20" t="inlineStr">
+        <is>
+          <t>Visit (optional link)</t>
+        </is>
+      </c>
+      <c r="E180" s="20" t="inlineStr">
+        <is>
+          <t>dropdown</t>
+        </is>
+      </c>
+      <c r="F180" s="20" t="inlineStr">
+        <is>
+          <t>Single column</t>
+        </is>
+      </c>
+      <c r="G180" s="20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H180" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I180" s="20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J180" s="20" t="inlineStr">
+        <is>
+          <t>Reference to a row in Visits</t>
+        </is>
+      </c>
+      <c r="K180" s="20" t="inlineStr">
+        <is>
+          <t>OPTIONAL — groups everything captured at one visit. Entries are valid without it (registry backfill).</t>
+        </is>
+      </c>
+      <c r="L180" s="20" t="inlineStr">
         <is>
           <t>PROPOSED (v3)</t>
         </is>

</xml_diff>